<commit_message>
allegedly patched edge case for parameter setting algorithm
</commit_message>
<xml_diff>
--- a/Excel_files/susswein_2025_model.xlsx
+++ b/Excel_files/susswein_2025_model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\udickman\pySNNAP\Excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB48E6E-8C16-427E-9ABE-CFA3B570228A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F1566A-8A1D-42C6-91B0-B20D59A6200C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="716" activeTab="5" xr2:uid="{F0735362-4961-42D4-9F52-DCA2C5A03203}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="716" xr2:uid="{F0735362-4961-42D4-9F52-DCA2C5A03203}"/>
   </bookViews>
   <sheets>
     <sheet name="Neu" sheetId="3" r:id="rId1"/>
@@ -3464,7 +3464,7 @@
     <col min="304" max="16384" width="9.1796875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:141" x14ac:dyDescent="0.35">
       <c r="D1" s="55" t="s">
         <v>86</v>
       </c>
@@ -3618,7 +3618,7 @@
       <c r="EJ1" s="154"/>
       <c r="EK1" s="155"/>
     </row>
-    <row r="2" spans="1:246" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:141" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E2" s="158" t="s">
         <v>88</v>
       </c>
@@ -3789,7 +3789,7 @@
       <c r="EJ2" s="150"/>
       <c r="EK2" s="152"/>
     </row>
-    <row r="3" spans="1:246" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:141" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="90" t="s">
         <v>0</v>
       </c>
@@ -4211,7 +4211,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A4" s="89" t="s">
         <v>166</v>
       </c>
@@ -4448,7 +4448,7 @@
       <c r="EJ4" s="146"/>
       <c r="EK4" s="148"/>
     </row>
-    <row r="5" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A5" s="89" t="s">
         <v>167</v>
       </c>
@@ -4685,7 +4685,7 @@
       <c r="EJ5" s="17"/>
       <c r="EK5" s="19"/>
     </row>
-    <row r="6" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A6" s="89" t="s">
         <v>168</v>
       </c>
@@ -4956,63 +4956,25 @@
       <c r="DH6" s="17"/>
       <c r="DI6" s="17"/>
       <c r="DJ6" s="19"/>
-      <c r="DK6" s="43">
-        <v>200</v>
-      </c>
-      <c r="DL6" s="17">
-        <v>1</v>
-      </c>
-      <c r="DM6" s="17">
-        <v>-35</v>
-      </c>
-      <c r="DN6" s="17">
-        <v>0</v>
-      </c>
-      <c r="DO6" s="17">
-        <v>-20</v>
-      </c>
-      <c r="DP6" s="17">
-        <v>2</v>
-      </c>
-      <c r="DQ6" s="17">
-        <v>1</v>
-      </c>
-      <c r="DR6" s="17">
-        <v>1.4E-2</v>
-      </c>
-      <c r="DS6" s="17">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="DT6" s="17">
-        <v>20</v>
-      </c>
-      <c r="DU6" s="17">
-        <v>7</v>
-      </c>
-      <c r="DV6" s="17">
-        <v>1</v>
-      </c>
-      <c r="DW6" s="17">
-        <v>-15</v>
-      </c>
-      <c r="DX6" s="17">
-        <v>-6</v>
-      </c>
-      <c r="DY6" s="17">
-        <v>1</v>
-      </c>
-      <c r="DZ6" s="17">
-        <v>0</v>
-      </c>
-      <c r="EA6" s="17">
-        <v>1000</v>
-      </c>
-      <c r="EB6" s="17">
-        <v>7</v>
-      </c>
-      <c r="EC6" s="17">
-        <v>1</v>
-      </c>
+      <c r="DK6" s="43"/>
+      <c r="DL6" s="17"/>
+      <c r="DM6" s="17"/>
+      <c r="DN6" s="17"/>
+      <c r="DO6" s="17"/>
+      <c r="DP6" s="17"/>
+      <c r="DQ6" s="17"/>
+      <c r="DR6" s="17"/>
+      <c r="DS6" s="17"/>
+      <c r="DT6" s="17"/>
+      <c r="DU6" s="17"/>
+      <c r="DV6" s="17"/>
+      <c r="DW6" s="17"/>
+      <c r="DX6" s="17"/>
+      <c r="DY6" s="17"/>
+      <c r="DZ6" s="17"/>
+      <c r="EA6" s="17"/>
+      <c r="EB6" s="17"/>
+      <c r="EC6" s="17"/>
       <c r="ED6" s="17"/>
       <c r="EE6" s="17"/>
       <c r="EF6" s="17"/>
@@ -5022,7 +4984,7 @@
       <c r="EJ6" s="17"/>
       <c r="EK6" s="19"/>
     </row>
-    <row r="7" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A7" s="89" t="s">
         <v>169</v>
       </c>
@@ -5273,107 +5235,83 @@
       <c r="DH7" s="17"/>
       <c r="DI7" s="17"/>
       <c r="DJ7" s="19"/>
-      <c r="DK7" s="43"/>
-      <c r="DL7" s="17"/>
-      <c r="DM7" s="17"/>
-      <c r="DN7" s="17"/>
-      <c r="DO7" s="17"/>
-      <c r="DP7" s="17"/>
-      <c r="DQ7" s="17"/>
-      <c r="DR7" s="17"/>
-      <c r="DS7" s="17"/>
-      <c r="DT7" s="17"/>
-      <c r="DU7" s="17"/>
-      <c r="DV7" s="17"/>
-      <c r="DW7" s="17"/>
-      <c r="DX7" s="17"/>
-      <c r="DY7" s="17"/>
-      <c r="DZ7" s="17"/>
-      <c r="EA7" s="17"/>
-      <c r="EB7" s="17"/>
-      <c r="EC7" s="17"/>
-      <c r="ED7" s="17"/>
-      <c r="EE7" s="17"/>
-      <c r="EF7" s="17"/>
-      <c r="EG7" s="17"/>
-      <c r="EH7" s="17"/>
+      <c r="DK7" s="43">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="DL7" s="17">
+        <v>3</v>
+      </c>
+      <c r="DM7" s="17">
+        <v>50</v>
+      </c>
+      <c r="DN7" s="17">
+        <v>0</v>
+      </c>
+      <c r="DO7" s="17">
+        <v>-48</v>
+      </c>
+      <c r="DP7" s="17">
+        <v>4</v>
+      </c>
+      <c r="DQ7" s="17">
+        <v>2</v>
+      </c>
+      <c r="DR7" s="17">
+        <v>0.16</v>
+      </c>
+      <c r="DS7" s="17">
+        <v>1.4999999999999999E-4</v>
+      </c>
+      <c r="DT7" s="17">
+        <v>-30</v>
+      </c>
+      <c r="DU7" s="17">
+        <v>4</v>
+      </c>
+      <c r="DV7" s="17">
+        <v>4</v>
+      </c>
+      <c r="DW7" s="17">
+        <v>-50</v>
+      </c>
+      <c r="DX7" s="17">
+        <v>-4</v>
+      </c>
+      <c r="DY7" s="17">
+        <v>4</v>
+      </c>
+      <c r="DZ7" s="17">
+        <v>0</v>
+      </c>
+      <c r="EA7" s="17">
+        <v>-57</v>
+      </c>
+      <c r="EB7" s="17">
+        <v>5</v>
+      </c>
+      <c r="EC7" s="17">
+        <v>2</v>
+      </c>
+      <c r="ED7" s="17">
+        <v>2</v>
+      </c>
+      <c r="EE7" s="17">
+        <v>0.2</v>
+      </c>
+      <c r="EF7" s="17">
+        <v>-44</v>
+      </c>
+      <c r="EG7" s="17">
+        <v>-3</v>
+      </c>
+      <c r="EH7" s="17">
+        <v>4</v>
+      </c>
       <c r="EI7" s="17"/>
       <c r="EJ7" s="17"/>
       <c r="EK7" s="19"/>
-      <c r="HO7" s="14">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="HP7" s="14">
-        <v>3</v>
-      </c>
-      <c r="HQ7" s="14">
-        <v>50</v>
-      </c>
-      <c r="HR7" s="14">
-        <v>0</v>
-      </c>
-      <c r="HS7" s="14">
-        <v>-48</v>
-      </c>
-      <c r="HT7" s="14">
-        <v>4</v>
-      </c>
-      <c r="HU7" s="14">
-        <v>2</v>
-      </c>
-      <c r="HV7" s="14">
-        <v>0.16</v>
-      </c>
-      <c r="HW7" s="14">
-        <v>1.4999999999999999E-4</v>
-      </c>
-      <c r="HX7" s="14">
-        <v>-30</v>
-      </c>
-      <c r="HY7" s="14">
-        <v>4</v>
-      </c>
-      <c r="HZ7" s="14">
-        <v>4</v>
-      </c>
-      <c r="IA7" s="14">
-        <v>-50</v>
-      </c>
-      <c r="IB7" s="14">
-        <v>-4</v>
-      </c>
-      <c r="IC7" s="14">
-        <v>4</v>
-      </c>
-      <c r="ID7" s="14">
-        <v>0</v>
-      </c>
-      <c r="IE7" s="14">
-        <v>-57</v>
-      </c>
-      <c r="IF7" s="14">
-        <v>5</v>
-      </c>
-      <c r="IG7" s="14">
-        <v>2</v>
-      </c>
-      <c r="IH7" s="14">
-        <v>2</v>
-      </c>
-      <c r="II7" s="14">
-        <v>0.2</v>
-      </c>
-      <c r="IJ7" s="14">
-        <v>-44</v>
-      </c>
-      <c r="IK7" s="14">
-        <v>-3</v>
-      </c>
-      <c r="IL7" s="14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:246" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A8" s="89" t="s">
         <v>170</v>
       </c>
@@ -5582,107 +5520,83 @@
       <c r="DH8" s="17"/>
       <c r="DI8" s="17"/>
       <c r="DJ8" s="19"/>
-      <c r="DK8" s="43"/>
-      <c r="DL8" s="17"/>
-      <c r="DM8" s="17"/>
-      <c r="DN8" s="17"/>
-      <c r="DO8" s="17"/>
-      <c r="DP8" s="17"/>
-      <c r="DQ8" s="17"/>
-      <c r="DR8" s="17"/>
-      <c r="DS8" s="17"/>
-      <c r="DT8" s="17"/>
-      <c r="DU8" s="17"/>
-      <c r="DV8" s="17"/>
-      <c r="DW8" s="17"/>
-      <c r="DX8" s="17"/>
-      <c r="DY8" s="17"/>
-      <c r="DZ8" s="17"/>
-      <c r="EA8" s="17"/>
-      <c r="EB8" s="17"/>
-      <c r="EC8" s="17"/>
-      <c r="ED8" s="17"/>
-      <c r="EE8" s="17"/>
-      <c r="EF8" s="17"/>
-      <c r="EG8" s="17"/>
-      <c r="EH8" s="17"/>
+      <c r="DK8" s="43">
+        <v>0.01</v>
+      </c>
+      <c r="DL8" s="17">
+        <v>3</v>
+      </c>
+      <c r="DM8" s="17">
+        <v>50</v>
+      </c>
+      <c r="DN8" s="17">
+        <v>0</v>
+      </c>
+      <c r="DO8" s="17">
+        <v>-48</v>
+      </c>
+      <c r="DP8" s="17">
+        <v>4</v>
+      </c>
+      <c r="DQ8" s="17">
+        <v>2</v>
+      </c>
+      <c r="DR8" s="17">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="DS8" s="17">
+        <v>0.04</v>
+      </c>
+      <c r="DT8" s="17">
+        <v>-56</v>
+      </c>
+      <c r="DU8" s="17">
+        <v>-3</v>
+      </c>
+      <c r="DV8" s="17">
+        <v>4</v>
+      </c>
+      <c r="DW8" s="17">
+        <v>-30</v>
+      </c>
+      <c r="DX8" s="17">
+        <v>-3</v>
+      </c>
+      <c r="DY8" s="17">
+        <v>4</v>
+      </c>
+      <c r="DZ8" s="17">
+        <v>0</v>
+      </c>
+      <c r="EA8" s="17">
+        <v>-56</v>
+      </c>
+      <c r="EB8" s="17">
+        <v>5</v>
+      </c>
+      <c r="EC8" s="17">
+        <v>2</v>
+      </c>
+      <c r="ED8" s="17">
+        <v>3</v>
+      </c>
+      <c r="EE8" s="17">
+        <v>0.05</v>
+      </c>
+      <c r="EF8" s="17">
+        <v>-40</v>
+      </c>
+      <c r="EG8" s="17">
+        <v>-2</v>
+      </c>
+      <c r="EH8" s="17">
+        <v>4</v>
+      </c>
       <c r="EI8" s="17"/>
       <c r="EJ8" s="17"/>
       <c r="EK8" s="19"/>
-      <c r="HO8" s="14">
-        <v>0.01</v>
-      </c>
-      <c r="HP8" s="14">
-        <v>3</v>
-      </c>
-      <c r="HQ8" s="14">
-        <v>50</v>
-      </c>
-      <c r="HR8" s="14">
-        <v>0</v>
-      </c>
-      <c r="HS8" s="14">
-        <v>-48</v>
-      </c>
-      <c r="HT8" s="14">
-        <v>4</v>
-      </c>
-      <c r="HU8" s="14">
-        <v>2</v>
-      </c>
-      <c r="HV8" s="14">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="HW8" s="14">
-        <v>0.04</v>
-      </c>
-      <c r="HX8" s="14">
-        <v>-56</v>
-      </c>
-      <c r="HY8" s="14">
-        <v>-3</v>
-      </c>
-      <c r="HZ8" s="14">
-        <v>4</v>
-      </c>
-      <c r="IA8" s="14">
-        <v>-30</v>
-      </c>
-      <c r="IB8" s="14">
-        <v>-3</v>
-      </c>
-      <c r="IC8" s="14">
-        <v>4</v>
-      </c>
-      <c r="ID8" s="14">
-        <v>0</v>
-      </c>
-      <c r="IE8" s="14">
-        <v>-56</v>
-      </c>
-      <c r="IF8" s="14">
-        <v>5</v>
-      </c>
-      <c r="IG8" s="14">
-        <v>2</v>
-      </c>
-      <c r="IH8" s="14">
-        <v>3</v>
-      </c>
-      <c r="II8" s="14">
-        <v>0.05</v>
-      </c>
-      <c r="IJ8" s="14">
-        <v>-40</v>
-      </c>
-      <c r="IK8" s="14">
-        <v>-2</v>
-      </c>
-      <c r="IL8" s="14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:246" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A9" s="89" t="s">
         <v>171</v>
       </c>
@@ -5919,7 +5833,7 @@
       <c r="EJ9" s="17"/>
       <c r="EK9" s="19"/>
     </row>
-    <row r="10" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A10" s="89" t="s">
         <v>172</v>
       </c>
@@ -6156,7 +6070,7 @@
       <c r="EJ10" s="17"/>
       <c r="EK10" s="19"/>
     </row>
-    <row r="11" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A11" s="89" t="s">
         <v>173</v>
       </c>
@@ -6443,63 +6357,25 @@
       <c r="DH11" s="17"/>
       <c r="DI11" s="17"/>
       <c r="DJ11" s="19"/>
-      <c r="DK11" s="43">
-        <v>200</v>
-      </c>
-      <c r="DL11" s="17">
-        <v>1</v>
-      </c>
-      <c r="DM11" s="17">
-        <v>-35</v>
-      </c>
-      <c r="DN11" s="17">
-        <v>0</v>
-      </c>
-      <c r="DO11" s="17">
-        <v>-20</v>
-      </c>
-      <c r="DP11" s="17">
-        <v>2</v>
-      </c>
-      <c r="DQ11" s="17">
-        <v>1</v>
-      </c>
-      <c r="DR11" s="17">
-        <v>1.4E-2</v>
-      </c>
-      <c r="DS11" s="17">
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="DT11" s="17">
-        <v>20</v>
-      </c>
-      <c r="DU11" s="17">
-        <v>7</v>
-      </c>
-      <c r="DV11" s="17">
-        <v>1</v>
-      </c>
-      <c r="DW11" s="17">
-        <v>-15</v>
-      </c>
-      <c r="DX11" s="17">
-        <v>-6</v>
-      </c>
-      <c r="DY11" s="17">
-        <v>1</v>
-      </c>
-      <c r="DZ11" s="17">
-        <v>0</v>
-      </c>
-      <c r="EA11" s="17">
-        <v>1000</v>
-      </c>
-      <c r="EB11" s="17">
-        <v>7</v>
-      </c>
-      <c r="EC11" s="17">
-        <v>1</v>
-      </c>
+      <c r="DK11" s="43"/>
+      <c r="DL11" s="17"/>
+      <c r="DM11" s="17"/>
+      <c r="DN11" s="17"/>
+      <c r="DO11" s="17"/>
+      <c r="DP11" s="17"/>
+      <c r="DQ11" s="17"/>
+      <c r="DR11" s="17"/>
+      <c r="DS11" s="17"/>
+      <c r="DT11" s="17"/>
+      <c r="DU11" s="17"/>
+      <c r="DV11" s="17"/>
+      <c r="DW11" s="17"/>
+      <c r="DX11" s="17"/>
+      <c r="DY11" s="17"/>
+      <c r="DZ11" s="17"/>
+      <c r="EA11" s="17"/>
+      <c r="EB11" s="17"/>
+      <c r="EC11" s="17"/>
       <c r="ED11" s="17"/>
       <c r="EE11" s="17"/>
       <c r="EF11" s="17"/>
@@ -6509,7 +6385,7 @@
       <c r="EJ11" s="17"/>
       <c r="EK11" s="19"/>
     </row>
-    <row r="12" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A12" s="89" t="s">
         <v>174</v>
       </c>
@@ -6760,107 +6636,83 @@
       <c r="DH12" s="17"/>
       <c r="DI12" s="17"/>
       <c r="DJ12" s="19"/>
-      <c r="DK12" s="43"/>
-      <c r="DL12" s="17"/>
-      <c r="DM12" s="17"/>
-      <c r="DN12" s="17"/>
-      <c r="DO12" s="17"/>
-      <c r="DP12" s="17"/>
-      <c r="DQ12" s="17"/>
-      <c r="DR12" s="17"/>
-      <c r="DS12" s="17"/>
-      <c r="DT12" s="17"/>
-      <c r="DU12" s="17"/>
-      <c r="DV12" s="17"/>
-      <c r="DW12" s="17"/>
-      <c r="DX12" s="17"/>
-      <c r="DY12" s="17"/>
-      <c r="DZ12" s="17"/>
-      <c r="EA12" s="17"/>
-      <c r="EB12" s="17"/>
-      <c r="EC12" s="17"/>
-      <c r="ED12" s="17"/>
-      <c r="EE12" s="17"/>
-      <c r="EF12" s="17"/>
-      <c r="EG12" s="17"/>
-      <c r="EH12" s="17"/>
+      <c r="DK12" s="43">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="DL12" s="17">
+        <v>3</v>
+      </c>
+      <c r="DM12" s="17">
+        <v>50</v>
+      </c>
+      <c r="DN12" s="17">
+        <v>0</v>
+      </c>
+      <c r="DO12" s="17">
+        <v>-48</v>
+      </c>
+      <c r="DP12" s="17">
+        <v>4</v>
+      </c>
+      <c r="DQ12" s="17">
+        <v>2</v>
+      </c>
+      <c r="DR12" s="17">
+        <v>0.16</v>
+      </c>
+      <c r="DS12" s="17">
+        <v>1.4999999999999999E-4</v>
+      </c>
+      <c r="DT12" s="17">
+        <v>-30</v>
+      </c>
+      <c r="DU12" s="17">
+        <v>4</v>
+      </c>
+      <c r="DV12" s="17">
+        <v>4</v>
+      </c>
+      <c r="DW12" s="17">
+        <v>-50</v>
+      </c>
+      <c r="DX12" s="17">
+        <v>-4</v>
+      </c>
+      <c r="DY12" s="17">
+        <v>4</v>
+      </c>
+      <c r="DZ12" s="17">
+        <v>0</v>
+      </c>
+      <c r="EA12" s="17">
+        <v>-57</v>
+      </c>
+      <c r="EB12" s="17">
+        <v>5</v>
+      </c>
+      <c r="EC12" s="17">
+        <v>2</v>
+      </c>
+      <c r="ED12" s="17">
+        <v>2</v>
+      </c>
+      <c r="EE12" s="17">
+        <v>0.2</v>
+      </c>
+      <c r="EF12" s="17">
+        <v>-44</v>
+      </c>
+      <c r="EG12" s="17">
+        <v>-3</v>
+      </c>
+      <c r="EH12" s="17">
+        <v>4</v>
+      </c>
       <c r="EI12" s="17"/>
       <c r="EJ12" s="17"/>
       <c r="EK12" s="19"/>
-      <c r="HO12" s="14">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="HP12" s="14">
-        <v>3</v>
-      </c>
-      <c r="HQ12" s="14">
-        <v>50</v>
-      </c>
-      <c r="HR12" s="14">
-        <v>0</v>
-      </c>
-      <c r="HS12" s="14">
-        <v>-48</v>
-      </c>
-      <c r="HT12" s="14">
-        <v>4</v>
-      </c>
-      <c r="HU12" s="14">
-        <v>2</v>
-      </c>
-      <c r="HV12" s="14">
-        <v>0.16</v>
-      </c>
-      <c r="HW12" s="14">
-        <v>1.4999999999999999E-4</v>
-      </c>
-      <c r="HX12" s="14">
-        <v>-30</v>
-      </c>
-      <c r="HY12" s="14">
-        <v>4</v>
-      </c>
-      <c r="HZ12" s="14">
-        <v>4</v>
-      </c>
-      <c r="IA12" s="14">
-        <v>-50</v>
-      </c>
-      <c r="IB12" s="14">
-        <v>-4</v>
-      </c>
-      <c r="IC12" s="14">
-        <v>4</v>
-      </c>
-      <c r="ID12" s="14">
-        <v>0</v>
-      </c>
-      <c r="IE12" s="14">
-        <v>-57</v>
-      </c>
-      <c r="IF12" s="14">
-        <v>5</v>
-      </c>
-      <c r="IG12" s="14">
-        <v>2</v>
-      </c>
-      <c r="IH12" s="14">
-        <v>2</v>
-      </c>
-      <c r="II12" s="14">
-        <v>0.2</v>
-      </c>
-      <c r="IJ12" s="14">
-        <v>-44</v>
-      </c>
-      <c r="IK12" s="14">
-        <v>-3</v>
-      </c>
-      <c r="IL12" s="14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:246" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A13" s="89" t="s">
         <v>175</v>
       </c>
@@ -7069,107 +6921,83 @@
       <c r="DH13" s="17"/>
       <c r="DI13" s="17"/>
       <c r="DJ13" s="19"/>
-      <c r="DK13" s="43"/>
-      <c r="DL13" s="17"/>
-      <c r="DM13" s="17"/>
-      <c r="DN13" s="17"/>
-      <c r="DO13" s="17"/>
-      <c r="DP13" s="17"/>
-      <c r="DQ13" s="17"/>
-      <c r="DR13" s="17"/>
-      <c r="DS13" s="17"/>
-      <c r="DT13" s="17"/>
-      <c r="DU13" s="17"/>
-      <c r="DV13" s="17"/>
-      <c r="DW13" s="17"/>
-      <c r="DX13" s="17"/>
-      <c r="DY13" s="17"/>
-      <c r="DZ13" s="17"/>
-      <c r="EA13" s="17"/>
-      <c r="EB13" s="17"/>
-      <c r="EC13" s="17"/>
-      <c r="ED13" s="17"/>
-      <c r="EE13" s="17"/>
-      <c r="EF13" s="17"/>
-      <c r="EG13" s="17"/>
-      <c r="EH13" s="17"/>
+      <c r="DK13" s="43">
+        <v>0.01</v>
+      </c>
+      <c r="DL13" s="17">
+        <v>3</v>
+      </c>
+      <c r="DM13" s="17">
+        <v>50</v>
+      </c>
+      <c r="DN13" s="17">
+        <v>0</v>
+      </c>
+      <c r="DO13" s="17">
+        <v>-48</v>
+      </c>
+      <c r="DP13" s="17">
+        <v>4</v>
+      </c>
+      <c r="DQ13" s="17">
+        <v>2</v>
+      </c>
+      <c r="DR13" s="17">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="DS13" s="17">
+        <v>0.04</v>
+      </c>
+      <c r="DT13" s="17">
+        <v>-56</v>
+      </c>
+      <c r="DU13" s="17">
+        <v>-3</v>
+      </c>
+      <c r="DV13" s="17">
+        <v>4</v>
+      </c>
+      <c r="DW13" s="17">
+        <v>-30</v>
+      </c>
+      <c r="DX13" s="17">
+        <v>-3</v>
+      </c>
+      <c r="DY13" s="17">
+        <v>4</v>
+      </c>
+      <c r="DZ13" s="17">
+        <v>0</v>
+      </c>
+      <c r="EA13" s="17">
+        <v>-56</v>
+      </c>
+      <c r="EB13" s="17">
+        <v>5</v>
+      </c>
+      <c r="EC13" s="17">
+        <v>2</v>
+      </c>
+      <c r="ED13" s="17">
+        <v>3</v>
+      </c>
+      <c r="EE13" s="17">
+        <v>0.05</v>
+      </c>
+      <c r="EF13" s="17">
+        <v>-40</v>
+      </c>
+      <c r="EG13" s="17">
+        <v>-2</v>
+      </c>
+      <c r="EH13" s="17">
+        <v>4</v>
+      </c>
       <c r="EI13" s="17"/>
       <c r="EJ13" s="17"/>
       <c r="EK13" s="19"/>
-      <c r="HO13" s="14">
-        <v>0.01</v>
-      </c>
-      <c r="HP13" s="14">
-        <v>3</v>
-      </c>
-      <c r="HQ13" s="14">
-        <v>50</v>
-      </c>
-      <c r="HR13" s="14">
-        <v>0</v>
-      </c>
-      <c r="HS13" s="14">
-        <v>-48</v>
-      </c>
-      <c r="HT13" s="14">
-        <v>4</v>
-      </c>
-      <c r="HU13" s="14">
-        <v>2</v>
-      </c>
-      <c r="HV13" s="14">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="HW13" s="14">
-        <v>0.04</v>
-      </c>
-      <c r="HX13" s="14">
-        <v>-56</v>
-      </c>
-      <c r="HY13" s="14">
-        <v>-3</v>
-      </c>
-      <c r="HZ13" s="14">
-        <v>4</v>
-      </c>
-      <c r="IA13" s="14">
-        <v>-30</v>
-      </c>
-      <c r="IB13" s="14">
-        <v>-3</v>
-      </c>
-      <c r="IC13" s="14">
-        <v>4</v>
-      </c>
-      <c r="ID13" s="14">
-        <v>0</v>
-      </c>
-      <c r="IE13" s="14">
-        <v>-56</v>
-      </c>
-      <c r="IF13" s="14">
-        <v>5</v>
-      </c>
-      <c r="IG13" s="14">
-        <v>2</v>
-      </c>
-      <c r="IH13" s="14">
-        <v>3</v>
-      </c>
-      <c r="II13" s="14">
-        <v>0.05</v>
-      </c>
-      <c r="IJ13" s="14">
-        <v>-40</v>
-      </c>
-      <c r="IK13" s="14">
-        <v>-2</v>
-      </c>
-      <c r="IL13" s="14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:246" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A14" s="89">
         <f>Neu!B14</f>
         <v>0</v>
@@ -7315,7 +7143,7 @@
       <c r="EJ14" s="17"/>
       <c r="EK14" s="19"/>
     </row>
-    <row r="15" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A15" s="89">
         <f>Neu!B15</f>
         <v>0</v>
@@ -7461,7 +7289,7 @@
       <c r="EJ15" s="17"/>
       <c r="EK15" s="19"/>
     </row>
-    <row r="16" spans="1:246" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:141" x14ac:dyDescent="0.35">
       <c r="A16" s="89">
         <f>Neu!B16</f>
         <v>0</v>
@@ -8856,49 +8684,6 @@
       <c r="EF25" s="23"/>
       <c r="EG25" s="23"/>
       <c r="EH25" s="23"/>
-      <c r="FE25" s="23"/>
-      <c r="FF25" s="23"/>
-      <c r="FG25" s="23"/>
-      <c r="FH25" s="23"/>
-      <c r="FI25" s="23"/>
-      <c r="FL25" s="23"/>
-      <c r="GL25" s="23"/>
-      <c r="HM25" s="23"/>
-      <c r="HO25" s="23"/>
-      <c r="HP25" s="23"/>
-      <c r="HQ25" s="23"/>
-      <c r="HR25" s="23"/>
-      <c r="HS25" s="23"/>
-      <c r="HT25" s="23"/>
-      <c r="HU25" s="23"/>
-      <c r="HV25" s="23"/>
-      <c r="HW25" s="23"/>
-      <c r="HX25" s="23"/>
-      <c r="HY25" s="23"/>
-      <c r="HZ25" s="23"/>
-      <c r="IA25" s="23"/>
-      <c r="IB25" s="23"/>
-      <c r="IC25" s="23"/>
-      <c r="ID25" s="23"/>
-      <c r="IE25" s="23"/>
-      <c r="IF25" s="23"/>
-      <c r="IG25" s="23"/>
-      <c r="IH25" s="23"/>
-      <c r="IP25" s="23"/>
-      <c r="IQ25" s="23"/>
-      <c r="IR25" s="23"/>
-      <c r="IS25" s="23"/>
-      <c r="IT25" s="23"/>
-      <c r="IU25" s="23"/>
-      <c r="IV25" s="23"/>
-      <c r="IW25" s="23"/>
-      <c r="IX25" s="23"/>
-      <c r="IY25" s="23"/>
-      <c r="IZ25" s="23"/>
-      <c r="JA25" s="23"/>
-      <c r="JB25" s="23"/>
-      <c r="JC25" s="23"/>
-      <c r="JD25" s="23"/>
     </row>
     <row r="26" spans="1:264" x14ac:dyDescent="0.35">
       <c r="G26" s="23"/>
@@ -10982,29 +10767,24 @@
       <formula>LEN(TRIM(FE26))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="FE25:FI25">
-    <cfRule type="notContainsBlanks" dxfId="31" priority="53">
-      <formula>LEN(TRIM(FE25))&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="FE27:FI27">
     <cfRule type="notContainsBlanks" dxfId="30" priority="51">
       <formula>LEN(TRIM(FE27))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="FL25:FL27">
+  <conditionalFormatting sqref="FL26:FL27">
     <cfRule type="notContainsBlanks" dxfId="29" priority="44">
-      <formula>LEN(TRIM(FL25))&gt;0</formula>
+      <formula>LEN(TRIM(FL26))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="GL25:GL27">
+  <conditionalFormatting sqref="GL26:GL27">
     <cfRule type="notContainsBlanks" dxfId="28" priority="75">
-      <formula>LEN(TRIM(GL25))&gt;0</formula>
+      <formula>LEN(TRIM(GL26))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="HM25:HM27">
+  <conditionalFormatting sqref="HM26:HM27">
     <cfRule type="notContainsBlanks" dxfId="27" priority="37">
-      <formula>LEN(TRIM(HM25))&gt;0</formula>
+      <formula>LEN(TRIM(HM26))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="HO29:HO31">
@@ -11012,29 +10792,24 @@
       <formula>LEN(TRIM(HO29))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="HO25:HU25 ID25:IH25">
-    <cfRule type="notContainsBlanks" dxfId="25" priority="147">
-      <formula>LEN(TRIM(HO25))&gt;0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="HO27:HU27 ID27:IH27">
     <cfRule type="notContainsBlanks" dxfId="24" priority="139">
       <formula>LEN(TRIM(HO27))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="HV25:IC27">
+  <conditionalFormatting sqref="HV26:IC27">
     <cfRule type="notContainsBlanks" dxfId="23" priority="24">
-      <formula>LEN(TRIM(HV25))&gt;0</formula>
+      <formula>LEN(TRIM(HV26))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="IP25:IV26">
+  <conditionalFormatting sqref="IP26:IV26">
     <cfRule type="notContainsBlanks" dxfId="22" priority="95">
-      <formula>LEN(TRIM(IP25))&gt;0</formula>
+      <formula>LEN(TRIM(IP26))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="IW25:JD27">
+  <conditionalFormatting sqref="IW26:JD27">
     <cfRule type="notContainsBlanks" dxfId="21" priority="101">
-      <formula>LEN(TRIM(IW25))&gt;0</formula>
+      <formula>LEN(TRIM(IW26))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>